<commit_message>
Add Pengsheng Design official vendor details
</commit_message>
<xml_diff>
--- a/data/whole-home-customization-vendors.public.xlsx
+++ b/data/whole-home-customization-vendors.public.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY11"/>
+  <dimension ref="A1:BD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,240 +435,265 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>official_website</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>official_phone</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>official_email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>official_wechat</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>showroom_locations</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>service_area</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>budget_positioning</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>design_style</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>materials</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>environmental_standard</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>typical_timeline</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>verification_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>verified_by</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>vendor_label</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>vendor_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>district</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>store_type</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>authorization</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>customer_segments</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>board_materials</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>recommended_boards</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>hardware</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>starting_price_projection</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>edge_band_material</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>edge_banding_process</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>edge_banding_equipment</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>cabinet_structure</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>cabinet_connectors_feet</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>measurement_design_fee</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>deposit_refund_policy</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>designer_team</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>rendering_cycle</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>outsourced_design</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>installation_team</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>damage_handling</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>floor_protection</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>aftersales_staff</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>warranty_policy</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>customization_cycle</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>retain_final_payment</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>payment_terms</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>creator_comment</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>strengths</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>caveats</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>source_name</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>source_author</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>source_date</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>source_page_or_rows</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>source_confidence</t>
         </is>
@@ -690,222 +715,227 @@
           <t>上海</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
         <is>
           <t>上海 徐汇区 上海市徐汇区龙启路258号（绿地汇中心）</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>中高预算</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>芙、芬萨、菲德来、水性科天、畔森ENF、模压板 柜体板建议：岭南木色海洋板、爱格、菲德莱、水性科天 油漆类产品基材：木皮、水性烤漆（欧松板、实木） 柜门板建议：爱格、可丽芙、菲德来、悦纹、靓时SPB</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>ENF；爱格；可丽芙；菲德莱；靓时；水性科天</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>一般为30天（工艺复杂特殊订单需延长5-10天） 交期较快，赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>门店一（白名单4.0门店）</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
         <is>
           <t>乐乐</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>上海市徐汇区龙启路258号（绿地汇中心）</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>徐汇区</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>写字楼工作室</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>上海唯一的靓时授权门店 水性科天</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>改善型客户/豪宅客户</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>芙、芬萨、菲德来、水性科天、畔森ENF、模压板 柜体板建议：岭南木色海洋板、爱格、菲德莱、水性科天 油漆类产品基材：木皮、水性烤漆（欧松板、实木） 柜门板建议：爱格、可丽芙、菲德来、悦纹、靓时SPB</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>板材品类 芙、芬萨、菲德来、水性科天、畔森ENF、模压板 柜体板建议：岭南木色海洋板、爱格、菲德莱、水性科天 油漆类产品基材：木皮、水性烤漆（欧松板、实木） 柜门板建议：爱格、可丽芙、菲德来、悦纹、靓时SPB</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>诺米，DTC，奥地利百隆，海蒂诗，萨里奇 国产五金优先考虑DTC</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>1350元/平</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>使用大厂封边带，类似华立、红棉花、兄奕、欧德雅等</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>封边设备 激光：豪迈激光封边机（璞缇工厂），PUR：豪迈PUR封边机 璞缇是国内全屋定制代工厂龙头企业，工艺水准较高</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>激光：豪迈激光封边机（璞缇工厂），PUR：豪迈PUR封边机 璞缇是国内全屋定制代工厂龙头企业，工艺水准较高</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>会根据实际情况而定，橱柜单元柜，衣柜不一定 建议有条件的客户上单元柜，更稳定耐用，单元柜用板量更大</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>国产四合一，二合一，无调整脚</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>当调整定金比例），再测量出图 会在免费设计的公司工作，因为工作强度和收入不成正比。建议根据自身需求选择</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>定金不退（可抵扣货款）</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>设计师2名</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>根据房屋大小，确定时间周期（1个星期左右） 常规水平</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>5名</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>根据订单总金额而定，金额大的会做地面保护，金额小的利润无法支持 地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板，一套房的地面保护成本大约大几</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>进行地面保护 百的水平，也是体现商家服务水平比较直观的点。</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>老板亲自跟售后</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>五金加木作（5年质保）</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>一般为30天（工艺复杂特殊订单需延长5-10天） 交期较快，赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>否 个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素，奈何太多人关心，还是放上来</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>定金+签合同全款下单</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>上海土著事业型女老板开的一家工作室，对材料认知非常到位，亲自全程跟单，交付快，服务体验</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>设计/整案能力较强；交付速度有优势；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；付款节点偏前，合同边界要写清；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>白名单商家信息表-上海汇总(1).pdf</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>pdf</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr">
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>page 1</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -927,222 +957,227 @@
           <t>上海</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>上海 宝山区 上海宝山区军工路</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制；整案/设计服务；硬装；软装</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>中预算/性价比</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>柜体板建议：爱格、菲德莱、吉林森工、兔宝宝 油漆类产品基材：红橡，樱桃木，胡桃木，北美黑胡桃，白蜡木，乌金 柜门板建议：爱格、菲德莱、可丽芙、善诺胜、福人精板 木</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>爱格；可丽芙；菲德莱；福人；兔宝宝</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>一般为45天工作日左右，油漆类60天左右 赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>门店二（白名单3.0门店）</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>葱姐</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>上海宝山区军工路</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>宝山区</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>整案设计公司：硬装、活动家具、全屋定制、软装</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>文信A类授权（爱格，飞德莱，善诺胜，可丽芙）福人精板、兔宝宝</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>刚需客户/改善型客户/别墅客户</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>柜体板建议：爱格、菲德莱、吉林森工、兔宝宝 油漆类产品基材：红橡，樱桃木，胡桃木，北美黑胡桃，白蜡木，乌金 柜门板建议：爱格、菲德莱、可丽芙、善诺胜、福人精板 木</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>精板F4星，兔宝宝enf级实木多层，模压板，吉林森工实木多层ENF级 板材品类 柜体板建议：爱格、菲德莱、吉林森工、兔宝宝 油漆类产品基材：红橡，樱桃木，胡桃木，北美黑胡桃，白蜡木，乌金 柜门板建议：爱格、菲德莱、可丽芙、善诺胜、福人精板 木</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>DTC，奥地利百隆 国产五金优先考虑DTC</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>1199/投影起</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>使用大厂封边带，类似华立、红棉花、兄奕、欧德雅等</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>艺优势里面最不值一提的一个。</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>德国豪迈激光封边机 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高，定位误差越小，五金使用越顺滑，使用寿命越长</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>单元柜 。IF调整脚的使用，也可以有效克服顶地不平的情况，使柜体安装效果更好。</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>三合一为主，部分文信25层板的工艺用四合一，进口IF连接件、调整脚</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>收费1000~3000元 会在免费设计的公司工作，因为工作强度和收入不成正比。建议根据自身需求选择</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>测量后不可退，方案不满意可退</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>室内设计师4名，全屋定制设计师6名，设计总监3名，图纸深化师1名</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>7-15天，根据设计师手里案子情况决定 常规水平</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AN3" t="inlineStr">
         <is>
           <t>稳定合作安装师傅4名</t>
         </is>
       </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AO3" t="inlineStr">
         <is>
           <t>地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板，一套房的地面保护成本大约大几</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AP3" t="inlineStr">
         <is>
           <t>会进行地面保护 百的水平，也是体现商家服务水平比较直观的点 有专职售后人员是售后问题快速响应的必备前提，特别是在出现不需要返厂的售后问题时，有专职</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>有，2名</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AR3" t="inlineStr">
         <is>
           <t>板材10年质保，国产五金5年，进口五金10年</t>
         </is>
       </c>
-      <c r="AN3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
         <is>
           <t>一般为45天工作日左右，油漆类60天左右 赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="AO3" t="inlineStr">
+      <c r="AT3" t="inlineStr">
         <is>
           <t>不留 个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素，奈何太多人关心，还是放上来</t>
         </is>
       </c>
-      <c r="AP3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t>定金+签合同付部分货款+复测完确定好最终方案付尾款</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
         <is>
           <t>上海诸多文信授权商家中综合实力较强且比较重视服务的一家店，有整案能力，老板靠谱实在</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AW3" t="inlineStr">
         <is>
           <t>设计/整案能力较强；性价比或入门价格有优势；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
+      <c r="AX3" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；工期不算短，需确认逾期责任；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AY3" t="inlineStr">
         <is>
           <t>白名单商家信息表-上海汇总(1).pdf</t>
         </is>
       </c>
-      <c r="AU3" t="inlineStr">
+      <c r="AZ3" t="inlineStr">
         <is>
           <t>pdf</t>
         </is>
       </c>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr">
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr">
         <is>
           <t>page 2</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr">
+      <c r="BD3" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -1164,222 +1199,227 @@
           <t>上海</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
         <is>
           <t>上海 徐汇区 上海市徐汇区宜山路欧雅广场</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>中预算/性价比</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>宝宝，爱格，芬萨，可丽芙，飞德莱，巴西博耐克，实木贴皮，烤漆门 柜体板建议：芦花板、新港仿生板、爱格、菲德莱 板，胡桃木，樱桃木，白橡木，油栎木，榆木，橡胶木等板材 柜门板建议：爱格、芦花、芬萨、可丽芙、博耐克 标配：DTC 图特，滑轨为图特全拉托底轨，进口五金：奥地利百隆，海</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>爱格；可丽芙；菲德莱；水性科天；福人</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>一般为45个工作日（特殊订单需延长） 赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>门店三（白名单3.0门店）</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>魏总</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>上海市徐汇区宜山路欧雅广场</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>徐汇区</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>写字楼工作室</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>福人精板，水性科天精板，芦花板精板，露水河精板，仿生板等国产板材。爱格，芬萨等进口板材</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>刚需客户，精装客户，毛坯客户，豪宅客户</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>宝宝，爱格，芬萨，可丽芙，飞德莱，巴西博耐克，实木贴皮，烤漆门 柜体板建议：芦花板、新港仿生板、爱格、菲德莱 板，胡桃木，樱桃木，白橡木，油栎木，榆木，橡胶木等板材 柜门板建议：爱格、芦花、芬萨、可丽芙、博耐克 标配：DTC 图特，滑轨为图特全拉托底轨，进口五金：奥地利百隆，海</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>板材品类 宝宝，爱格，芬萨，可丽芙，飞德莱，巴西博耐克，实木贴皮，烤漆门 柜体板建议：芦花板、新港仿生板、爱格、菲德莱 板，胡桃木，樱桃木，白橡木，油栎木，榆木，橡胶木等板材 柜门板建议：爱格、芦花、芬萨、可丽芙、博耐克 标配：DTC 图特，滑轨为图特全拉托底轨，进口五金：奥地利百隆，海</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>国产优先DTC 蒂诗，萨里奇</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>1080/投影</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>封边 封边工艺</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>封边设备 极东的PUR 极东是国产设备龙头，做柜体足够用了</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>极东的PUR 极东是国产设备龙头，做柜体足够用了</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>柜体</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>三合一连接件 无调整脚 （橱柜有调整脚）</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>图 会在免费设计的公司工作，因为工作强度和收入不成正比。建议根据自身需求选择</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>方案不满意可退一半，客户自愿取消合作不退</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>设计师6名</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>两周起</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AN4" t="inlineStr">
         <is>
           <t>8名</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AO4" t="inlineStr">
         <is>
           <t>根据订单总金额而定，金额大的会做地面保护，金额小的利润无法支持 地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板，一套房的地面保护成本大约大几</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr">
+      <c r="AP4" t="inlineStr">
         <is>
           <t>进行地面保护 百的水平，也是体现商家服务水平比较直观的点 有专职售后人员是售后问题快速响应的必备前提，特别是在出现不需要返厂的售后问题时，有专职</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr">
+      <c r="AQ4" t="inlineStr">
         <is>
           <t>三名</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr">
+      <c r="AR4" t="inlineStr">
         <is>
           <t>五年质保，终身维护</t>
         </is>
       </c>
-      <c r="AN4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
         <is>
           <t>一般为45个工作日（特殊订单需延长） 赔付标准需协商明确</t>
         </is>
       </c>
-      <c r="AO4" t="inlineStr">
+      <c r="AT4" t="inlineStr">
         <is>
           <t>协商 个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素，奈何太多人关心，还是放上来</t>
         </is>
       </c>
-      <c r="AP4" t="inlineStr">
+      <c r="AU4" t="inlineStr">
         <is>
           <t>定金+签合同付90%货款+货到现场付剩下尾款</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr">
+      <c r="AV4" t="inlineStr">
         <is>
           <t>白名单老店，服务水平提高的非常快，近一年0投诉，性价比很高</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AW4" t="inlineStr">
         <is>
           <t>设计/整案能力较强；性价比或入门价格有优势；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；工期不算短，需确认逾期责任；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AY4" t="inlineStr">
         <is>
           <t>白名单商家信息表-上海汇总(1).pdf</t>
         </is>
       </c>
-      <c r="AU4" t="inlineStr">
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>pdf</t>
         </is>
       </c>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr">
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr">
         <is>
           <t>page 3</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr">
+      <c r="BD4" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -1403,220 +1443,249 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>杭州 拱墅区 杭州市拱墅区影天像素园</t>
+          <t>https://pengshengdesign.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>全屋定制；柜体定制；整案/设计服务</t>
+          <t>+86 153-7203-0216</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>info@pengshengdesign.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tanya0324</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>拱墅工作室：浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室；临平木作展厅：浙江省杭州市临平区顺风路536号32幢101室</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>杭州 拱墅区 临平区；拱墅工作室；临平木作展厅；浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>全屋定制；柜体定制；整案/设计服务；私宅设计；软装；全屋定制木作</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>中高预算/高配置</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>免漆板材： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时 油漆板材： 天然木皮。混油</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>爱格；可丽芙；靓时</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>一般为60个工作日（特殊订单需延长）</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>门店一（白名单4.0门店）</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>澎升设计 Pengsheng Design</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>马老师</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>杭州市拱墅区影天像素园</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>拱墅区</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>设计公司</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>设计公司/工作室/木作展厅</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
         <is>
           <t>惟嘉工厂授权</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>改善型客户、平层、别墅客户</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>免漆板材： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时 油漆板材： 天然木皮。混油</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 亿维雅、 韩伟乐 柜门板建议： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>奥地利百隆</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>1500/投影</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>ABS/PP</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>激光 / PUR</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>豪迈激光封边机</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>单元柜</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>进口IF四合一、 调整脚</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>全案设计收设计费/定制设计收预估价10%</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>服务后定金不退 ，方案做到满意为止</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>设计师8名、 建模1名</t>
         </is>
       </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AL5" t="inlineStr">
         <is>
           <t>15天左右</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AM5" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AN5" t="inlineStr">
         <is>
           <t>8名</t>
         </is>
       </c>
-      <c r="AJ5" t="inlineStr">
+      <c r="AO5" t="inlineStr">
         <is>
           <t>重新生产</t>
         </is>
       </c>
-      <c r="AK5" t="inlineStr">
+      <c r="AP5" t="inlineStr">
         <is>
           <t>保护</t>
         </is>
       </c>
-      <c r="AL5" t="inlineStr">
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>1名</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>五金5年 ，木作5年</t>
         </is>
       </c>
-      <c r="AN5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
         <is>
           <t>一般为60个工作日（特殊订单需延长）</t>
         </is>
       </c>
-      <c r="AO5" t="inlineStr">
+      <c r="AT5" t="inlineStr">
         <is>
           <t>不留尾款</t>
         </is>
       </c>
-      <c r="AP5" t="inlineStr">
+      <c r="AU5" t="inlineStr">
         <is>
           <t>定金+签合同付清尾款</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>设计师创作能力强，管理能力突出，有pmp证书、擅长全案设计、整案输出；可以溯源、可做的工艺类型比较多；服务能力与目标客群匹配度较高， 改善客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 亿维雅、 韩伟乐 柜门板建议： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时；高配封边带，ABS/PP封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州最高；配置较高，通常破损不严重的地方大多数商家采取补漆处理；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>设计师创作能力强，管理能力突出，有pmp证书、擅长全案设计、整案输出；可以溯源、可做的工艺类型比较多；服务能力与目标客群匹配度较高， 改善客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 亿维雅、 韩伟乐 柜门板建议： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时；高配封边带，ABS/PP封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州最高；配置较高，通常破损不严重的地方大多数商家采取补漆处理；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来；官网补充：澎升设计 Pengsheng Design，定位为杭州本土化设计公司，强调私宅设计、产品设计、软装与全屋定制服务；官网列出全屋定制木作、拱墅工作室和临平木作展厅。</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
         <is>
           <t>设计/整案能力较强；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS5" t="inlineStr">
+      <c r="AX5" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；工期不算短，需确认逾期责任；付款节点偏前，合同边界要写清；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>白名单商家信息表-杭州汇总(2).xlsx</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>白名单商家信息表-杭州汇总(2).xlsx；pengshengdesign.com 官网</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
         <is>
           <t>xlsx</t>
         </is>
       </c>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr">
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr">
         <is>
           <t>rows 2-34</t>
         </is>
       </c>
-      <c r="AY5" t="inlineStr">
+      <c r="BD5" t="inlineStr">
         <is>
           <t>high</t>
         </is>
@@ -1638,222 +1707,227 @@
           <t>杭州</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
         <is>
           <t>杭州 西湖区 杭州市西湖区古墩路888号红星美凯龙至尊茂</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>中高预算/高配置</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>免漆板材： 爱格、 可丽芙、 菲德莱、 善诺胜、 文信木恪 油漆板材： 天然木皮</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>爱格；可丽芙；菲德莱</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>一般为60个工作日（特殊订单需延长）</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>门店二（白名单4.0门店）</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
         <is>
           <t>孙老师</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>杭州市西湖区古墩路888号红星美凯龙至尊茂</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>西湖区</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>商场店</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>文信木特专卖店</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>改善型客户</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>免漆板材： 爱格、 可丽芙、 菲德莱、 善诺胜、 文信木恪 油漆板材： 天然木皮</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 菲德莱、 文信木恪 柜门板建议： 爱格、 可丽芙、 菲德莱、 善诺胜</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>奥地利百隆</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>1500/投影</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>ABS/PP</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>激光 / PUR</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>豪迈激光封边机</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>单元柜</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>进口IF四合一、 调整脚</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>先收定金： 10000元 。 再出效果图</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>服务后定金不退 ，方案做到满意为止</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr">
+      <c r="AK6" t="inlineStr">
         <is>
           <t>设计师8名、 建模1名</t>
         </is>
       </c>
-      <c r="AG6" t="inlineStr">
+      <c r="AL6" t="inlineStr">
         <is>
           <t>15天左右</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AN6" t="inlineStr">
         <is>
           <t>8名</t>
         </is>
       </c>
-      <c r="AJ6" t="inlineStr">
+      <c r="AO6" t="inlineStr">
         <is>
           <t>重新生产</t>
         </is>
       </c>
-      <c r="AK6" t="inlineStr">
+      <c r="AP6" t="inlineStr">
         <is>
           <t>保护</t>
         </is>
       </c>
-      <c r="AL6" t="inlineStr">
+      <c r="AQ6" t="inlineStr">
         <is>
           <t>1名</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr">
+      <c r="AR6" t="inlineStr">
         <is>
           <t>五金10年 ，木作1年</t>
         </is>
       </c>
-      <c r="AN6" t="inlineStr">
+      <c r="AS6" t="inlineStr">
         <is>
           <t>一般为60个工作日（特殊订单需延长）</t>
         </is>
       </c>
-      <c r="AO6" t="inlineStr">
+      <c r="AT6" t="inlineStr">
         <is>
           <t>不留尾款</t>
         </is>
       </c>
-      <c r="AP6" t="inlineStr">
+      <c r="AU6" t="inlineStr">
         <is>
           <t>定金+签合同付清尾款</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr">
+      <c r="AV6" t="inlineStr">
         <is>
           <t>白名单好评度和稳定性最高的一家店， 五年0投诉 ， 团队管理水平在定制行业里面算是比较高的 了， 主打一个稳 。 有整案能力，支持局改 ，有软装部；浙江省提货量最大的文信经销商，全国排前五 ， 实力没的说；服务能力与目标客群匹配度较高， 改善客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 菲德莱、 文信木恪 柜门板建议： 爱格、 可丽芙、 菲德莱、 善诺胜；高配封边带，ABS/PP封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州天花板水平（高定除外）；配置较高，通常破损不严重的地方大多数商家采取补漆处理；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AW6" t="inlineStr">
         <is>
           <t>设计/整案能力较强；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
+      <c r="AX6" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；工期不算短，需确认逾期责任；付款节点偏前，合同边界要写清；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT6" t="inlineStr">
+      <c r="AY6" t="inlineStr">
         <is>
           <t>白名单商家信息表-杭州汇总(2).xlsx</t>
         </is>
       </c>
-      <c r="AU6" t="inlineStr">
+      <c r="AZ6" t="inlineStr">
         <is>
           <t>xlsx</t>
         </is>
       </c>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr">
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr">
         <is>
           <t>rows 35-67</t>
         </is>
       </c>
-      <c r="AY6" t="inlineStr">
+      <c r="BD6" t="inlineStr">
         <is>
           <t>high</t>
         </is>
@@ -1875,222 +1949,227 @@
           <t>杭州</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
         <is>
           <t>杭州 西湖区 杭州市西湖区古墩路701号红星美凯龙世博家居生活广场</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>中预算/性价比</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>免漆类板材品牌： 爱格、 善诺胜、 可丽芙、 菲德来、 文信绿芯、 福人、 岭南木色ENF级海洋板、 靓时、 奥凯奇 油漆类产品基材： 红橡 ，樱桃木，榆木 ， 胡桃木（木皮）</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>ENF；爱格；可丽芙；靓时；福人</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>合同75个工作日（不可抗拒因素顺延）</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>门店三（白名单4.0门店）</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
         <is>
           <t>陈老师</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>杭州市西湖区古墩路701号红星美凯龙世博家居生活广场</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>西湖区</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>商场店</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>文信A</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>改善型/豪宅</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>免漆类板材品牌： 爱格、 善诺胜、 可丽芙、 菲德来、 文信绿芯、 福人、 岭南木色ENF级海洋板、 靓时、 奥凯奇 油漆类产品基材： 红橡 ，樱桃木，榆木 ， 胡桃木（木皮）</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 岭南木色、 靓时、 菲德莱、 文信绿芯 柜门板建议： 爱格、 可丽芙、 靓时、 福人精板、 善诺胜</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>标配： 奥利百隆 一字铰链 托底轨钢板抽（DTC 海蒂诗等可选）</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>1199</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>abs</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>激光 / PUR</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>进口板， 豪迈激光封边机</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>单元柜</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>意大利IF调整脚 JW12连接件</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>先收定金， 后测量</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>方案满意为止， 定金不可退</t>
         </is>
       </c>
-      <c r="AF7" t="inlineStr">
+      <c r="AK7" t="inlineStr">
         <is>
           <t>设计师6名 ， 软装设计师3名 ，硬装设计师1名</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AL7" t="inlineStr">
         <is>
           <t>10-15天</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>自有设计师</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr">
+      <c r="AN7" t="inlineStr">
         <is>
           <t>自有安装班组4组</t>
         </is>
       </c>
-      <c r="AJ7" t="inlineStr">
+      <c r="AO7" t="inlineStr">
         <is>
           <t>重新生产 ，修补（视情况而定）</t>
         </is>
       </c>
-      <c r="AK7" t="inlineStr">
+      <c r="AP7" t="inlineStr">
         <is>
           <t>安装前铺设</t>
         </is>
       </c>
-      <c r="AL7" t="inlineStr">
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>2名</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr">
+      <c r="AR7" t="inlineStr">
         <is>
           <t>柜体5年五金10年（国产五金、 油漆产品另议）</t>
         </is>
       </c>
-      <c r="AN7" t="inlineStr">
+      <c r="AS7" t="inlineStr">
         <is>
           <t>合同75个工作日（不可抗拒因素顺延）</t>
         </is>
       </c>
-      <c r="AO7" t="inlineStr">
+      <c r="AT7" t="inlineStr">
         <is>
           <t>协商</t>
         </is>
       </c>
-      <c r="AP7" t="inlineStr">
+      <c r="AU7" t="inlineStr">
         <is>
           <t>定金+签合同付部分货款+货到现场付全款（尾款协商）</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AV7" t="inlineStr">
         <is>
           <t>杭州文信经销商里面性价比最高的一家（非最低价） ，服务配置基本对齐拜哈木特 ，但是该店有美 的集团补贴支持，运营成本更低，售价也比拜哈木特要低一些；服务能力与目标客群匹配度较高， 改善型客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 岭南木色、 靓时、 菲德莱、 文信绿芯 柜门板建议： 爱格、 可丽芙、 靓时、 福人精板、 善诺胜；国产优先DTC ，但是做文信的柜体最好用百隆；高配封边带，ABS封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州天花板水平（高定除外）；常规操作；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr">
+      <c r="AW7" t="inlineStr">
         <is>
           <t>设计/整案能力较强；性价比或入门价格有优势；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
+      <c r="AX7" t="inlineStr">
         <is>
           <t>定金退款规则需提前确认；工期不算短，需确认逾期责任；付款节点偏前，合同边界要写清；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr">
+      <c r="AY7" t="inlineStr">
         <is>
           <t>白名单商家信息表-杭州汇总(2).xlsx</t>
         </is>
       </c>
-      <c r="AU7" t="inlineStr">
+      <c r="AZ7" t="inlineStr">
         <is>
           <t>xlsx</t>
         </is>
       </c>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr">
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr">
         <is>
           <t>rows 68-100</t>
         </is>
       </c>
-      <c r="AY7" t="inlineStr">
+      <c r="BD7" t="inlineStr">
         <is>
           <t>high</t>
         </is>
@@ -2112,222 +2191,227 @@
           <t>杭州</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
         <is>
           <t>杭州 滨江区 滨江区</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>全屋定制；柜体定制</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>性价比/预算友好</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
         <is>
           <t>爱格 福人 兔宝宝 千年舟 大王椰 悦纹 可丽芙 欧卡菲 橡胶木 新西 兰松木 亿维雅 烤漆 混油 水性漆</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>爱格；可丽芙；福人；兔宝宝</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>定制周期根据板材品牌而定 库存内15到25天 非库存内 35到45天 逾期 赔付合同金额3%</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>门店四（白名单3.0门店）</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
         <is>
           <t>向总</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>滨江区</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>滨江区</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>工厂店</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>爱格 福人 兔宝宝 千年舟 大王椰 悦纹</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>刚需改善和部分豪宅</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>爱格 福人 兔宝宝 千年舟 大王椰 悦纹 可丽芙 欧卡菲 橡胶木 新西 兰松木 亿维雅 烤漆 混油 水性漆</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 欧卡菲、 新西兰松木 柜门板建议： 爱格、 可丽芙、 悦纹、 福人</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>标配DTC或者悍高 可选择升级百隆 海蒂诗 补差每投影100</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>980</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>均有 不同板材厂家配置</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>激光 pur (门板体系内纯色免费升级激光)</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AF8" t="inlineStr">
         <is>
           <t>豪迈 豪德</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AG8" t="inlineStr">
         <is>
           <t>多为单元柜 具体会因实际设计而定</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AH8" t="inlineStr">
         <is>
           <t>国产三合一 二合一 要求可升级进口IF五金连接件</t>
         </is>
       </c>
-      <c r="AD8" t="inlineStr">
+      <c r="AI8" t="inlineStr">
         <is>
           <t>先收取定金后量尺 5000定金 投影多会适当调整定金金额</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AJ8" t="inlineStr">
         <is>
           <t>可退 方案不满意扣除工本费1500元其余全退</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr">
+      <c r="AK8" t="inlineStr">
         <is>
           <t>设计4名</t>
         </is>
       </c>
-      <c r="AG8" t="inlineStr">
+      <c r="AL8" t="inlineStr">
         <is>
           <t>7天</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr">
+      <c r="AM8" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AN8" t="inlineStr">
         <is>
           <t>两组安装师傅 每组配备2个师傅一个小工共计6名</t>
         </is>
       </c>
-      <c r="AJ8" t="inlineStr">
+      <c r="AO8" t="inlineStr">
         <is>
           <t>影响结构 破损无法使用等重新生产 小磕碰美容师修复</t>
         </is>
       </c>
-      <c r="AK8" t="inlineStr">
+      <c r="AP8" t="inlineStr">
         <is>
           <t>单值超过6万进场前会进行地面保护 低于会使用板材包装材料进行铺装 保护</t>
         </is>
       </c>
-      <c r="AL8" t="inlineStr">
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>1个</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AR8" t="inlineStr">
         <is>
           <t>进口五年 国产三年</t>
         </is>
       </c>
-      <c r="AN8" t="inlineStr">
+      <c r="AS8" t="inlineStr">
         <is>
           <t>定制周期根据板材品牌而定 库存内15到25天 非库存内 35到45天 逾期 赔付合同金额3%</t>
         </is>
       </c>
-      <c r="AO8" t="inlineStr">
+      <c r="AT8" t="inlineStr">
         <is>
           <t>不留 如强烈需要会留1到3千元</t>
         </is>
       </c>
-      <c r="AP8" t="inlineStr">
+      <c r="AU8" t="inlineStr">
         <is>
           <t>定金 签合同95货款 发货时全额付清</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AV8" t="inlineStr">
         <is>
           <t>自有工厂，体量比较大 ，授权齐全， 自有团队配置到位 ， 改补速度快 。 惟嘉爱格在杭州最大的授权 商之一；服务能力与目标客群匹配度较高， 刚需型客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 欧卡菲、 新西兰松木 柜门板建议： 爱格、 可丽芙、 悦纹、 福人；国产优先DTC；非异形件尽量选择ABS封边带 ，环保更有确定性 。 异形件必须使用PVC封边带的， 务必使用大品牌产品；建议有条件的客户上单元柜 ，更稳定耐用 ， 单元柜用板量更大；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州中等水平；常规水平；杭州中上水平；常规操作；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr">
+      <c r="AW8" t="inlineStr">
         <is>
           <t>设计/整案能力较强；交付速度有优势；性价比或入门价格有优势；售后响应配置较明确；柜体/封边工艺配置较完整</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
+      <c r="AX8" t="inlineStr">
         <is>
           <t>付款节点偏前，合同边界要写清；预算门槛可能偏高</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr">
+      <c r="AY8" t="inlineStr">
         <is>
           <t>白名单商家信息表-杭州汇总(2).xlsx</t>
         </is>
       </c>
-      <c r="AU8" t="inlineStr">
+      <c r="AZ8" t="inlineStr">
         <is>
           <t>xlsx</t>
         </is>
       </c>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr">
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr">
         <is>
           <t>rows 101-133</t>
         </is>
       </c>
-      <c r="AY8" t="inlineStr">
+      <c r="BD8" t="inlineStr">
         <is>
           <t>high</t>
         </is>
@@ -2349,42 +2433,42 @@
           <t>杭州</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>杭州</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>全屋定制；柜体定制</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>杭州</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>全屋定制；柜体定制</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>猴哥/大V白名单资料</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>小红书博主列出商家</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>DCEO</t>
-        </is>
-      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>猴哥/大V白名单资料</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>小红书博主列出商家</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>DCEO</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
@@ -2408,43 +2492,48 @@
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr">
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr">
         <is>
           <t>来自小红书笔记《后续来了，增加两家重量级全屋定制探店记录》。正文提到新增 DCEO 和马库住建工厂；图片/表格明细未完整结构化抽取。原文评分权重：口碑5%、展厅5%、设计25%、价格/性价比25%、服务20%、工艺20%。案例条件：二手房，投影面积40~42㎡，中古风；柜体考虑国产或者进口二线品牌，柜门使用爱格。</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
+      <c r="AW9" t="inlineStr">
         <is>
           <t>博主探店笔记明确列出；可作为杭州候选商家线索</t>
         </is>
       </c>
-      <c r="AS9" t="inlineStr">
+      <c r="AX9" t="inlineStr">
         <is>
           <t>缺少结构化价格、地址、材料、工艺、售后等字段；需补具体截图/原表或二次核验后再强推荐</t>
         </is>
       </c>
-      <c r="AT9" t="inlineStr">
+      <c r="AY9" t="inlineStr">
         <is>
           <t>后续来了，增加两家重量级全屋定制探店记录</t>
         </is>
       </c>
-      <c r="AU9" t="inlineStr">
+      <c r="AZ9" t="inlineStr">
         <is>
           <t>xiaohongshu_url</t>
         </is>
       </c>
-      <c r="AV9" t="inlineStr">
+      <c r="BA9" t="inlineStr">
         <is>
           <t>呼伦贝尔的风</t>
         </is>
       </c>
-      <c r="AW9" t="inlineStr">
+      <c r="BB9" t="inlineStr">
         <is>
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="AX9" t="inlineStr"/>
-      <c r="AY9" t="inlineStr">
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr">
         <is>
           <t>low</t>
         </is>
@@ -2475,21 +2564,21 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>小红书探店笔记</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>DCEO；马库住建工厂</t>
-        </is>
-      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>小红书探店笔记</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>DCEO；马库住建工厂</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
@@ -2513,43 +2602,48 @@
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr">
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr">
         <is>
           <t>后续来了，增加两家重量级全屋定制探店记录。作者提到新增 DCEO 和马库住建工厂。评分权重：口碑5%、展厅5%、设计25%、价格/性价比25%、服务20%、工艺20%。案例条件：二手房，投影面积40~42㎡，中古风；柜体考虑国产或者进口二线品牌，柜门使用爱格。原文提示资料为个人主观感受，只可大致参考，不作为决策依据。</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr">
+      <c r="AW10" t="inlineStr">
         <is>
           <t>提供评分维度和权重；可作为用户自评/推荐排序参考；补充两个杭州候选商家线索</t>
         </is>
       </c>
-      <c r="AS10" t="inlineStr">
+      <c r="AX10" t="inlineStr">
         <is>
           <t>网页正文未包含图片表格明细；需补截图或原始表格后才能精确入库</t>
         </is>
       </c>
-      <c r="AT10" t="inlineStr">
+      <c r="AY10" t="inlineStr">
         <is>
           <t>后续来了，增加两家重量级全屋定制探店记录</t>
         </is>
       </c>
-      <c r="AU10" t="inlineStr">
+      <c r="AZ10" t="inlineStr">
         <is>
           <t>xiaohongshu_url</t>
         </is>
       </c>
-      <c r="AV10" t="inlineStr">
+      <c r="BA10" t="inlineStr">
         <is>
           <t>呼伦贝尔的风</t>
         </is>
       </c>
-      <c r="AW10" t="inlineStr">
+      <c r="BB10" t="inlineStr">
         <is>
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="AX10" t="inlineStr"/>
-      <c r="AY10" t="inlineStr">
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -2580,16 +2674,16 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>小红书搜索入口</t>
-        </is>
-      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>小红书搜索入口</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2614,39 +2708,44 @@
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
-      <c r="AQ11" t="inlineStr">
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr">
         <is>
           <t>小红书搜索入口，关键词为“杭州全屋定制排名”。网页可见标题和筛选入口，但未暴露具体笔记卡片、作者、日期或正文。该来源适合作为后续检索入口，不适合作为单独商家推荐证据。后续可从该搜索页挑选具体笔记 URL、截图或原始表格后再拆分入库。</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr">
+      <c r="AW11" t="inlineStr">
         <is>
           <t>可持续发现杭州全屋定制排名/避坑/探店相关笔记；适合后续人工筛选具体来源</t>
         </is>
       </c>
-      <c r="AS11" t="inlineStr">
+      <c r="AX11" t="inlineStr">
         <is>
           <t>搜索页没有稳定披露具体笔记内容；不能直接用于推荐结论；需二次打开具体笔记或保存截图</t>
         </is>
       </c>
-      <c r="AT11" t="inlineStr">
+      <c r="AY11" t="inlineStr">
         <is>
           <t>杭州全屋定制排名 - 小红书搜索</t>
         </is>
       </c>
-      <c r="AU11" t="inlineStr">
+      <c r="AZ11" t="inlineStr">
         <is>
           <t>xiaohongshu_search_url</t>
         </is>
       </c>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr">
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="AX11" t="inlineStr"/>
-      <c r="AY11" t="inlineStr">
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr">
         <is>
           <t>low</t>
         </is>
@@ -2663,7 +2762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2713,15 +2812,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>official_website</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Public official website when known.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>official_phone</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -2729,7 +2832,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>budget_positioning</t>
+          <t>official_email</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -2737,7 +2840,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>design_style</t>
+          <t>official_wechat</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -2745,15 +2848,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>materials</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>showroom_locations</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Public showroom/workspace addresses when known.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>environmental_standard</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -2761,7 +2868,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>typical_timeline</t>
+          <t>scope</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -2769,7 +2876,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>verification_date</t>
+          <t>budget_positioning</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -2777,7 +2884,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>verified_by</t>
+          <t>design_style</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -2785,7 +2892,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>vendor_label</t>
+          <t>materials</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -2793,19 +2900,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>vendor_name</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Formal vendor name when known; blank means the source only gave a label/contact.</t>
-        </is>
-      </c>
+          <t>environmental_standard</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>contact_person</t>
+          <t>typical_timeline</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -2813,7 +2916,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>verification_date</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -2821,7 +2924,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>verified_by</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -2829,7 +2932,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>store_type</t>
+          <t>vendor_label</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -2837,15 +2940,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>authorization</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>vendor_name</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Formal vendor name when known; blank means the source only gave a label/contact.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>customer_segments</t>
+          <t>contact_person</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -2853,7 +2960,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>board_materials</t>
+          <t>address</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -2861,7 +2968,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>recommended_boards</t>
+          <t>district</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -2869,7 +2976,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>store_type</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -2877,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>starting_price_projection</t>
+          <t>authorization</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -2885,7 +2992,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>edge_band_material</t>
+          <t>customer_segments</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -2893,7 +3000,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>edge_banding_process</t>
+          <t>board_materials</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -2901,7 +3008,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>edge_banding_equipment</t>
+          <t>recommended_boards</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -2909,7 +3016,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cabinet_structure</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -2917,7 +3024,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cabinet_connectors_feet</t>
+          <t>starting_price_projection</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -2925,7 +3032,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>measurement_design_fee</t>
+          <t>edge_band_material</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -2933,7 +3040,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>deposit_refund_policy</t>
+          <t>edge_banding_process</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -2941,7 +3048,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>designer_team</t>
+          <t>edge_banding_equipment</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -2949,7 +3056,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>rendering_cycle</t>
+          <t>cabinet_structure</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -2957,7 +3064,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>outsourced_design</t>
+          <t>cabinet_connectors_feet</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -2965,7 +3072,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>installation_team</t>
+          <t>measurement_design_fee</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -2973,7 +3080,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>damage_handling</t>
+          <t>deposit_refund_policy</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -2981,7 +3088,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>floor_protection</t>
+          <t>designer_team</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -2989,7 +3096,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>aftersales_staff</t>
+          <t>rendering_cycle</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -2997,7 +3104,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>warranty_policy</t>
+          <t>outsourced_design</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -3005,7 +3112,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>customization_cycle</t>
+          <t>installation_team</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -3013,7 +3120,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>retain_final_payment</t>
+          <t>damage_handling</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -3021,7 +3128,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>payment_terms</t>
+          <t>floor_protection</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -3029,19 +3136,15 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>creator_comment</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Summarized creator/source comment; verify before publishing as final advice.</t>
-        </is>
-      </c>
+          <t>aftersales_staff</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>strengths</t>
+          <t>warranty_policy</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -3049,19 +3152,15 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>caveats</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Known fit limits or verification reminders.</t>
-        </is>
-      </c>
+          <t>customization_cycle</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>source_name</t>
+          <t>retain_final_payment</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -3069,7 +3168,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>payment_terms</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -3077,15 +3176,19 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>source_author</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
+          <t>creator_comment</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Summarized creator/source comment; verify before publishing as final advice.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>source_date</t>
+          <t>strengths</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -3093,18 +3196,62 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>source_page_or_rows</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
+          <t>caveats</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Known fit limits or verification reminders.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>source_author</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>source_date</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>source_page_or_rows</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>source_confidence</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>high/medium/low confidence in structured extraction completeness.</t>
         </is>

</xml_diff>

<commit_message>
Correct Pengsheng official contact details
</commit_message>
<xml_diff>
--- a/data/whole-home-customization-vendors.public.xlsx
+++ b/data/whole-home-customization-vendors.public.xlsx
@@ -1448,27 +1448,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+86 153-7203-0216</t>
+          <t>+86 13735800742</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>info@pengshengdesign.com</t>
+          <t>m5637379@gmail.com</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tanya0324</t>
+          <t>PengshengDesign</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>拱墅工作室：浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室；临平木作展厅：浙江省杭州市临平区顺风路536号32幢101室</t>
+          <t>拱墅工作室：杭州市拱墅区影天像素园澎升设计；临平全屋定制木作展厅：杭州市临平区元星大厦澎升设计</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>杭州 拱墅区 临平区；拱墅工作室；临平木作展厅；浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室</t>
+          <t>杭州 拱墅区 临平区；拱墅工作室；临平全屋定制木作展厅；杭州市拱墅区影天像素园澎升设计；杭州市临平区元星大厦澎升设计</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1497,7 +1497,11 @@
           <t>一般为60个工作日（特殊订单需延长）</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>猴哥/大V白名单资料</t>
@@ -1520,7 +1524,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区祥茂路2号影天像素园5幢A座402室</t>
+          <t>杭州市拱墅区影天像素园澎升设计</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1655,7 +1659,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>设计师创作能力强，管理能力突出，有pmp证书、擅长全案设计、整案输出；可以溯源、可做的工艺类型比较多；服务能力与目标客群匹配度较高， 改善客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 亿维雅、 韩伟乐 柜门板建议： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时；高配封边带，ABS/PP封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州最高；配置较高，通常破损不严重的地方大多数商家采取补漆处理；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来；官网补充：澎升设计 Pengsheng Design，定位为杭州本土化设计公司，强调私宅设计、产品设计、软装与全屋定制服务；官网列出全屋定制木作、拱墅工作室和临平木作展厅。</t>
+          <t>设计师创作能力强，管理能力突出，有pmp证书、擅长全案设计、整案输出；可以溯源、可做的工艺类型比较多；服务能力与目标客群匹配度较高， 改善客户满意度和转介绍率高；猴哥推荐搭配（基于板材物理性能和饰面美观度考虑） 柜体板建议： 爱格、 亿维雅、 韩伟乐 柜门板建议： 爱格、 可丽芙、 亿维雅、 韩伟乐、 靓时；高配封边带，ABS/PP封边带的环保水平较高 ，价格也高于PVC封边带；文信标配工艺， 虽然互联网平台上提及文信主要是说他们激光封边优秀 ，个人认为这仅仅是文信工 艺优势里面最不值一提的一个。 文信工艺最有价值的地方是柜体而非柜门，全套进口加工设备（而非仅仅是进口封边机） 带来的不 仅是封边的美观度，还有开孔的精密度，这对于提高柜体的稳定性和耐用性至关重要。 同时，越高端的五金对定位开孔的精度要求越高 ， 定位误差越小， 五金使用越顺滑 ，使用寿命越长 。 IF调整脚的使用， 也可以有效克服顶地不平的情况 ， 使柜体安装效果更好。 进口连接件和调整脚 ，这是大多数国内代工厂没有应用的。；虽然市场上有很多免费测量、 设计的公司 ，但是另一个市场现实也同样存在 ， 就是优秀的设计师不 会在免费设计的公司工作 ， 因为工作强度和收入不成正比 。 建议根据自身需求选择；杭州较高水平；常规水平；杭州最高；配置较高，通常破损不严重的地方大多数商家采取补漆处理；地面保护主要是防止柜子安装过程中的划伤，特别是保护木地板 ， 一套房的地面保护成本大约大几 百的水平， 也是体现商家服务水平比较直观的点；有专职售后人员是售后问题快速响应的必备前提 ，特别是在出现不需要返厂的售后问题时， 有专职 售后人员的门店能给客户更好的服务体验；个人认为是否留尾款不属于判断全屋定制是否靠谱的核心因素， 奈何太多人关心 ，还是放上来；官网补充：澎升设计 Pengsheng Design，定位为杭州本土化设计公司，强调私宅设计、产品设计、软装与全屋定制服务；官网列出木作/全屋定制、拱墅工作室和临平全屋定制木作展厅。</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">

</xml_diff>